<commit_message>
0.9.0 Add some conclusion codes and document append operation
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusion-code-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusion-code-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.8.1</t>
+    <t>0.9.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-02</t>
+    <t>2026-06-05</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -123,7 +123,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>Level</t>
@@ -189,10 +189,19 @@
     <t>1006</t>
   </si>
   <si>
-    <t>Øyelegeundersøkelse (grunnet diabetisk retinopati)</t>
-  </si>
-  <si>
-    <t>Patient is leaving the screening program and should be referred to an ophthalmologist for further examination due to findings of diabetic retinopathy.</t>
+    <t>Oppfølging i programmet settes på vent</t>
+  </si>
+  <si>
+    <t>Participation in the screening program is put on hold.</t>
+  </si>
+  <si>
+    <t>1007</t>
+  </si>
+  <si>
+    <t>Oppfølging i programmet avsluttes</t>
+  </si>
+  <si>
+    <t>Patient is discharged from the screening program.</t>
   </si>
 </sst>
 </file>
@@ -502,7 +511,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -603,6 +612,20 @@
         <v>59</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="C8" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s" s="2">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>